<commit_message>
Audit and fix all GitHub Actions workflows with requirements.txt and permissions
</commit_message>
<xml_diff>
--- a/load_test_report.xlsx
+++ b/load_test_report.xlsx
@@ -568,7 +568,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>47363</t>
+          <t>57329</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>787.89 req/sec</t>
+          <t>954.38 req/sec</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>91.18 ms</t>
+          <t>95.67 ms</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.21 ms</t>
+          <t>1.09 ms</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>1630.32 ms</t>
+          <t>1762.37 ms</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>528.88 ms</t>
+          <t>522.07 ms</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>69.71%</t>
+          <t>75.03%</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">

</xml_diff>